<commit_message>
added John Mason's video and Carmen's PDFs
</commit_message>
<xml_diff>
--- a/UConnBleedBlue/wwwroot/Data/Players.xlsx
+++ b/UConnBleedBlue/wwwroot/Data/Players.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\UConnBleedBlue\UConnBleedBlue\wwwroot\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA8C0F6-576F-40D8-9E2E-5EFFAB5CC538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42277B30-3352-4A19-946C-EEDE87FBB192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2325" windowWidth="38640" windowHeight="21120" xr2:uid="{4F83266A-41F9-4FA3-9290-1EB5622BBFC1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="673">
   <si>
     <t>Demers, Kenny</t>
   </si>
@@ -1517,9 +1517,6 @@
     <t>Total Donations</t>
   </si>
   <si>
-    <t>Extra Tickets Needed</t>
-  </si>
-  <si>
     <t>Silva,John</t>
   </si>
   <si>
@@ -2055,6 +2052,9 @@
   </si>
   <si>
     <t>Horvath,Howard</t>
+  </si>
+  <si>
+    <t>To ME Cash App</t>
   </si>
 </sst>
 </file>
@@ -2153,7 +2153,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2211,6 +2211,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2609,9 +2612,12 @@
       <c r="E4" s="11" t="b">
         <v>1</v>
       </c>
+      <c r="F4" s="23">
+        <v>100</v>
+      </c>
       <c r="J4" s="6">
         <f>SUM(F2:F329)</f>
-        <v>12050</v>
+        <v>12150</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -2650,9 +2656,6 @@
       <c r="E6" s="11" t="b">
         <v>1</v>
       </c>
-      <c r="J6" s="1" t="s">
-        <v>493</v>
-      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -2667,10 +2670,6 @@
       <c r="E7" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="J7" s="1">
-        <f>SUM(G2:G329)</f>
-        <v>3</v>
-      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -2683,7 +2682,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -2706,7 +2705,7 @@
         <v>100</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -2720,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2743,7 +2742,7 @@
         <v>250</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -2762,13 +2761,16 @@
       <c r="E12" s="11" t="b">
         <v>1</v>
       </c>
+      <c r="J12" s="14" t="s">
+        <v>672</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>531</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>532</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>533</v>
       </c>
       <c r="C13" s="1">
         <v>1987</v>
@@ -2782,7 +2784,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>485</v>
@@ -2822,10 +2824,10 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>647</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>648</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>649</v>
       </c>
       <c r="C16" s="1">
         <v>1996</v>
@@ -2890,10 +2892,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>655</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>656</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>657</v>
       </c>
       <c r="C20" s="1">
         <v>1995</v>
@@ -2935,10 +2937,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>642</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>643</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>644</v>
       </c>
       <c r="C23" s="1">
         <v>1982</v>
@@ -2949,7 +2951,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>341</v>
@@ -2963,10 +2965,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>498</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>499</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>500</v>
       </c>
       <c r="C25" s="1">
         <v>1977</v>
@@ -2977,10 +2979,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>585</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>586</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>587</v>
       </c>
       <c r="C26" s="1">
         <v>2004</v>
@@ -3053,10 +3055,10 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C31" s="1">
         <v>2017</v>
@@ -3081,10 +3083,10 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>504</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>505</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>506</v>
       </c>
       <c r="C33" s="1">
         <v>1998</v>
@@ -3106,10 +3108,10 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>547</v>
+      </c>
+      <c r="B35" s="3" t="s">
         <v>548</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>549</v>
       </c>
       <c r="C35" s="1">
         <v>1993</v>
@@ -3182,10 +3184,10 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>630</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>631</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>632</v>
       </c>
       <c r="E40" s="1" t="b">
         <v>0</v>
@@ -3213,10 +3215,10 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="E42" s="14" t="b">
         <v>1</v>
@@ -3224,7 +3226,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>293</v>
@@ -3241,10 +3243,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>541</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>542</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>543</v>
       </c>
       <c r="C44" s="1">
         <v>1973</v>
@@ -3255,10 +3257,10 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>502</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>503</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>504</v>
       </c>
       <c r="C45" s="1">
         <v>1981</v>
@@ -3407,14 +3409,14 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B55" s="3"/>
       <c r="C55" s="1">
         <v>2025</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="E55" s="1" t="b">
         <v>0</v>
@@ -3560,10 +3562,10 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>523</v>
+      </c>
+      <c r="B65" s="3" t="s">
         <v>524</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>525</v>
       </c>
       <c r="E65" s="1" t="b">
         <v>0</v>
@@ -3602,7 +3604,7 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B68" s="15"/>
       <c r="E68" s="14" t="b">
@@ -3628,10 +3630,10 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="B70" s="3" t="s">
         <v>650</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>651</v>
       </c>
       <c r="C70" s="1">
         <v>2002</v>
@@ -3656,10 +3658,10 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="B72" s="3" t="s">
         <v>528</v>
-      </c>
-      <c r="B72" s="3" t="s">
-        <v>529</v>
       </c>
       <c r="C72" s="1">
         <v>1994</v>
@@ -3670,10 +3672,10 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="B73" s="3" t="s">
         <v>582</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>583</v>
       </c>
       <c r="C73" s="1">
         <v>2000</v>
@@ -3718,13 +3720,13 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="B76" s="3" t="s">
         <v>511</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="D76" s="8" t="s">
         <v>512</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>513</v>
       </c>
       <c r="E76" s="1" t="b">
         <v>0</v>
@@ -3749,10 +3751,10 @@
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="B78" s="3" t="s">
         <v>591</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>592</v>
       </c>
       <c r="C78" s="1">
         <v>2015</v>
@@ -3831,10 +3833,10 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>561</v>
+      </c>
+      <c r="B83" s="3" t="s">
         <v>562</v>
-      </c>
-      <c r="B83" s="3" t="s">
-        <v>563</v>
       </c>
       <c r="C83" s="1">
         <v>1983</v>
@@ -3856,10 +3858,10 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>587</v>
+      </c>
+      <c r="B85" s="3" t="s">
         <v>588</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>589</v>
       </c>
       <c r="C85" s="1">
         <v>2009</v>
@@ -3887,10 +3889,10 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>559</v>
+      </c>
+      <c r="B87" s="7" t="s">
         <v>560</v>
-      </c>
-      <c r="B87" s="7" t="s">
-        <v>561</v>
       </c>
       <c r="C87" s="1">
         <v>1985</v>
@@ -3912,7 +3914,7 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>415</v>
@@ -3929,10 +3931,10 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C90" s="1">
         <v>1981</v>
@@ -4011,10 +4013,10 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>557</v>
+      </c>
+      <c r="B95" s="3" t="s">
         <v>558</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>559</v>
       </c>
       <c r="C95" s="1">
         <v>2003</v>
@@ -4025,10 +4027,10 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>640</v>
+      </c>
+      <c r="B96" s="3" t="s">
         <v>641</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>642</v>
       </c>
       <c r="C96" s="1">
         <v>1980</v>
@@ -4087,10 +4089,10 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>644</v>
+      </c>
+      <c r="B100" s="3" t="s">
         <v>645</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>646</v>
       </c>
       <c r="C100" s="1">
         <v>1990</v>
@@ -4129,10 +4131,10 @@
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>623</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>624</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>625</v>
       </c>
       <c r="C103" s="1">
         <v>1978</v>
@@ -4141,7 +4143,7 @@
         <v>1</v>
       </c>
       <c r="J103" s="8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
@@ -4158,7 +4160,7 @@
         <v>0</v>
       </c>
       <c r="J104" s="11" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
@@ -4166,7 +4168,7 @@
         <v>197</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="C105" s="1">
         <v>1982</v>
@@ -4178,7 +4180,7 @@
         <v>1</v>
       </c>
       <c r="J105" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
@@ -4198,12 +4200,12 @@
         <v>500</v>
       </c>
       <c r="J106" s="13" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B107" s="3"/>
       <c r="F107" s="18">
@@ -4227,6 +4229,9 @@
       <c r="F108" s="17">
         <v>50</v>
       </c>
+      <c r="J108" s="14" t="s">
+        <v>672</v>
+      </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
@@ -4247,10 +4252,10 @@
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>533</v>
+      </c>
+      <c r="B110" s="3" t="s">
         <v>534</v>
-      </c>
-      <c r="B110" s="3" t="s">
-        <v>535</v>
       </c>
       <c r="C110" s="1">
         <v>2021</v>
@@ -4298,10 +4303,10 @@
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
+        <v>549</v>
+      </c>
+      <c r="B113" s="3" t="s">
         <v>550</v>
-      </c>
-      <c r="B113" s="3" t="s">
-        <v>551</v>
       </c>
       <c r="C113" s="1">
         <v>1988</v>
@@ -4340,10 +4345,10 @@
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
+        <v>506</v>
+      </c>
+      <c r="B116" s="3" t="s">
         <v>507</v>
-      </c>
-      <c r="B116" s="3" t="s">
-        <v>508</v>
       </c>
       <c r="C116" s="1">
         <v>1988</v>
@@ -4354,10 +4359,10 @@
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
+        <v>595</v>
+      </c>
+      <c r="B117" s="3" t="s">
         <v>596</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>597</v>
       </c>
       <c r="C117" s="1">
         <v>2004</v>
@@ -4368,10 +4373,10 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
+        <v>597</v>
+      </c>
+      <c r="B118" s="3" t="s">
         <v>598</v>
-      </c>
-      <c r="B118" s="3" t="s">
-        <v>599</v>
       </c>
       <c r="C118" s="1">
         <v>2008</v>
@@ -4382,10 +4387,10 @@
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>579</v>
+      </c>
+      <c r="B119" s="3" t="s">
         <v>580</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>581</v>
       </c>
       <c r="C119" s="1">
         <v>1963</v>
@@ -4402,10 +4407,10 @@
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>519</v>
+      </c>
+      <c r="B120" s="3" t="s">
         <v>520</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>521</v>
       </c>
       <c r="C120" s="1">
         <v>1976</v>
@@ -4475,10 +4480,10 @@
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>551</v>
+      </c>
+      <c r="B125" s="3" t="s">
         <v>552</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>553</v>
       </c>
       <c r="C125" s="1">
         <v>1979</v>
@@ -4534,10 +4539,10 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>545</v>
+      </c>
+      <c r="B129" s="3" t="s">
         <v>546</v>
-      </c>
-      <c r="B129" s="3" t="s">
-        <v>547</v>
       </c>
       <c r="C129" s="1">
         <v>1970</v>
@@ -4548,10 +4553,10 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
+        <v>515</v>
+      </c>
+      <c r="B130" s="3" t="s">
         <v>516</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>517</v>
       </c>
       <c r="C130" s="1">
         <v>2009</v>
@@ -4607,7 +4612,7 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B134" s="3"/>
       <c r="E134" s="1" t="b">
@@ -4658,10 +4663,10 @@
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
+        <v>563</v>
+      </c>
+      <c r="B138" s="3" t="s">
         <v>564</v>
-      </c>
-      <c r="B138" s="3" t="s">
-        <v>565</v>
       </c>
       <c r="E138" s="1" t="b">
         <v>0</v>
@@ -4686,7 +4691,7 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>476</v>
@@ -4720,10 +4725,10 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
+        <v>638</v>
+      </c>
+      <c r="B142" s="3" t="s">
         <v>639</v>
-      </c>
-      <c r="B142" s="3" t="s">
-        <v>640</v>
       </c>
       <c r="C142" s="1">
         <v>1987</v>
@@ -4745,10 +4750,10 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>599</v>
+      </c>
+      <c r="B144" s="3" t="s">
         <v>600</v>
-      </c>
-      <c r="B144" s="3" t="s">
-        <v>601</v>
       </c>
       <c r="C144" s="1">
         <v>1988</v>
@@ -4759,10 +4764,10 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
+        <v>625</v>
+      </c>
+      <c r="B145" s="3" t="s">
         <v>626</v>
-      </c>
-      <c r="B145" s="3" t="s">
-        <v>627</v>
       </c>
       <c r="C145" s="1">
         <v>1980</v>
@@ -4807,10 +4812,10 @@
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
+        <v>592</v>
+      </c>
+      <c r="B148" s="7" t="s">
         <v>593</v>
-      </c>
-      <c r="B148" s="7" t="s">
-        <v>594</v>
       </c>
       <c r="C148" s="1">
         <v>2021</v>
@@ -4936,7 +4941,7 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>336</v>
@@ -4964,10 +4969,10 @@
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
+        <v>508</v>
+      </c>
+      <c r="B159" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="B159" s="3" t="s">
-        <v>510</v>
       </c>
       <c r="C159" s="1">
         <v>1968</v>
@@ -4984,7 +4989,7 @@
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B160" s="3"/>
       <c r="C160" s="1">
@@ -5171,10 +5176,10 @@
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
+        <v>611</v>
+      </c>
+      <c r="B172" s="3" t="s">
         <v>612</v>
-      </c>
-      <c r="B172" s="3" t="s">
-        <v>613</v>
       </c>
       <c r="C172" s="1">
         <v>1998</v>
@@ -5202,10 +5207,10 @@
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>574</v>
+      </c>
+      <c r="B174" s="3" t="s">
         <v>575</v>
-      </c>
-      <c r="B174" s="3" t="s">
-        <v>576</v>
       </c>
       <c r="C174" s="1">
         <v>2002</v>
@@ -5264,10 +5269,10 @@
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
+        <v>555</v>
+      </c>
+      <c r="B178" s="3" t="s">
         <v>556</v>
-      </c>
-      <c r="B178" s="3" t="s">
-        <v>557</v>
       </c>
       <c r="C178" s="1">
         <v>1975</v>
@@ -5402,10 +5407,10 @@
     </row>
     <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C187" s="1">
         <v>1976</v>
@@ -5462,7 +5467,7 @@
         <v>0</v>
       </c>
       <c r="J190" s="8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="191" spans="1:10" x14ac:dyDescent="0.25">
@@ -5479,7 +5484,7 @@
         <v>0</v>
       </c>
       <c r="J191" s="11" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="192" spans="1:10" x14ac:dyDescent="0.25">
@@ -5499,7 +5504,7 @@
         <v>50</v>
       </c>
       <c r="J192" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="193" spans="1:10" x14ac:dyDescent="0.25">
@@ -5516,7 +5521,7 @@
         <v>0</v>
       </c>
       <c r="J193" s="13" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="194" spans="1:10" x14ac:dyDescent="0.25">
@@ -5535,13 +5540,16 @@
       <c r="E194" s="11" t="b">
         <v>1</v>
       </c>
+      <c r="J194" s="14" t="s">
+        <v>672</v>
+      </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
+        <v>583</v>
+      </c>
+      <c r="B195" s="3" t="s">
         <v>584</v>
-      </c>
-      <c r="B195" s="3" t="s">
-        <v>585</v>
       </c>
       <c r="C195" s="1">
         <v>1996</v>
@@ -5563,10 +5571,10 @@
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
+        <v>571</v>
+      </c>
+      <c r="B197" s="3" t="s">
         <v>572</v>
-      </c>
-      <c r="B197" s="3" t="s">
-        <v>573</v>
       </c>
       <c r="C197" s="1">
         <v>1985</v>
@@ -5659,10 +5667,10 @@
     </row>
     <row r="203" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
+        <v>577</v>
+      </c>
+      <c r="B203" s="3" t="s">
         <v>578</v>
-      </c>
-      <c r="B203" s="3" t="s">
-        <v>579</v>
       </c>
       <c r="E203" s="11" t="b">
         <v>1</v>
@@ -5715,7 +5723,7 @@
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B207" s="3" t="s">
         <v>342</v>
@@ -5822,10 +5830,10 @@
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
+        <v>613</v>
+      </c>
+      <c r="B214" s="3" t="s">
         <v>614</v>
-      </c>
-      <c r="B214" s="3" t="s">
-        <v>615</v>
       </c>
       <c r="C214" s="1">
         <v>1973</v>
@@ -5890,10 +5898,10 @@
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
+        <v>636</v>
+      </c>
+      <c r="B218" s="3" t="s">
         <v>637</v>
-      </c>
-      <c r="B218" s="3" t="s">
-        <v>638</v>
       </c>
       <c r="C218" s="1">
         <v>1995</v>
@@ -5938,10 +5946,10 @@
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
+        <v>653</v>
+      </c>
+      <c r="B221" s="3" t="s">
         <v>654</v>
-      </c>
-      <c r="B221" s="3" t="s">
-        <v>655</v>
       </c>
       <c r="C221" s="1">
         <v>1978</v>
@@ -5983,10 +5991,10 @@
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="C224" s="1">
         <v>2010</v>
@@ -5997,10 +6005,10 @@
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
+        <v>513</v>
+      </c>
+      <c r="B225" s="3" t="s">
         <v>514</v>
-      </c>
-      <c r="B225" s="3" t="s">
-        <v>515</v>
       </c>
       <c r="C225" s="1">
         <v>2004</v>
@@ -6028,10 +6036,10 @@
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C227" s="1">
         <v>2003</v>
@@ -6101,10 +6109,10 @@
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
+        <v>569</v>
+      </c>
+      <c r="B232" s="3" t="s">
         <v>570</v>
-      </c>
-      <c r="B232" s="3" t="s">
-        <v>571</v>
       </c>
       <c r="E232" s="1" t="b">
         <v>0</v>
@@ -6287,10 +6295,10 @@
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
+        <v>609</v>
+      </c>
+      <c r="B244" s="3" t="s">
         <v>610</v>
-      </c>
-      <c r="B244" s="3" t="s">
-        <v>611</v>
       </c>
       <c r="C244" s="1">
         <v>1985</v>
@@ -6332,10 +6340,10 @@
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
+        <v>535</v>
+      </c>
+      <c r="B247" s="3" t="s">
         <v>536</v>
-      </c>
-      <c r="B247" s="3" t="s">
-        <v>537</v>
       </c>
       <c r="E247" s="1" t="b">
         <v>0</v>
@@ -6377,10 +6385,10 @@
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
+        <v>539</v>
+      </c>
+      <c r="B250" s="3" t="s">
         <v>540</v>
-      </c>
-      <c r="B250" s="3" t="s">
-        <v>541</v>
       </c>
       <c r="C250" s="1">
         <v>1981</v>
@@ -6436,10 +6444,10 @@
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
+        <v>601</v>
+      </c>
+      <c r="B254" s="3" t="s">
         <v>602</v>
-      </c>
-      <c r="B254" s="3" t="s">
-        <v>603</v>
       </c>
       <c r="C254" s="1">
         <v>1990</v>
@@ -6450,10 +6458,10 @@
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
+        <v>496</v>
+      </c>
+      <c r="B255" s="3" t="s">
         <v>497</v>
-      </c>
-      <c r="B255" s="3" t="s">
-        <v>498</v>
       </c>
       <c r="C255" s="1">
         <v>1993</v>
@@ -6478,10 +6486,10 @@
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
+        <v>628</v>
+      </c>
+      <c r="B257" s="3" t="s">
         <v>629</v>
-      </c>
-      <c r="B257" s="3" t="s">
-        <v>630</v>
       </c>
       <c r="C257" s="1">
         <v>1962</v>
@@ -6574,10 +6582,10 @@
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
+        <v>616</v>
+      </c>
+      <c r="B263" s="3" t="s">
         <v>617</v>
-      </c>
-      <c r="B263" s="3" t="s">
-        <v>618</v>
       </c>
       <c r="C263" s="1">
         <v>1998</v>
@@ -6616,7 +6624,7 @@
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B266" s="3"/>
       <c r="C266" s="1">
@@ -6648,10 +6656,10 @@
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
+        <v>657</v>
+      </c>
+      <c r="B268" s="3" t="s">
         <v>658</v>
-      </c>
-      <c r="B268" s="3" t="s">
-        <v>659</v>
       </c>
       <c r="C268" s="1">
         <v>1995</v>
@@ -6662,10 +6670,10 @@
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
+        <v>659</v>
+      </c>
+      <c r="B269" s="3" t="s">
         <v>660</v>
-      </c>
-      <c r="B269" s="3" t="s">
-        <v>661</v>
       </c>
       <c r="C269" s="1">
         <v>1995</v>
@@ -6707,10 +6715,10 @@
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
+        <v>565</v>
+      </c>
+      <c r="B272" s="3" t="s">
         <v>566</v>
-      </c>
-      <c r="B272" s="3" t="s">
-        <v>567</v>
       </c>
       <c r="C272" s="1">
         <v>2020</v>
@@ -6721,10 +6729,10 @@
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
+        <v>493</v>
+      </c>
+      <c r="B273" s="3" t="s">
         <v>494</v>
-      </c>
-      <c r="B273" s="3" t="s">
-        <v>495</v>
       </c>
       <c r="E273" s="1" t="b">
         <v>0</v>
@@ -6783,10 +6791,10 @@
     </row>
     <row r="277" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
+        <v>634</v>
+      </c>
+      <c r="B277" s="3" t="s">
         <v>635</v>
-      </c>
-      <c r="B277" s="3" t="s">
-        <v>636</v>
       </c>
       <c r="C277" s="1">
         <v>1971</v>
@@ -6884,10 +6892,10 @@
     </row>
     <row r="284" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
+        <v>517</v>
+      </c>
+      <c r="B284" s="3" t="s">
         <v>518</v>
-      </c>
-      <c r="B284" s="3" t="s">
-        <v>519</v>
       </c>
       <c r="C284" s="1">
         <v>1973</v>
@@ -6994,10 +7002,10 @@
     </row>
     <row r="291" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
+        <v>521</v>
+      </c>
+      <c r="B291" s="3" t="s">
         <v>522</v>
-      </c>
-      <c r="B291" s="3" t="s">
-        <v>523</v>
       </c>
       <c r="C291" s="1">
         <v>1974</v>
@@ -7068,7 +7076,7 @@
         <v>50</v>
       </c>
       <c r="J295" s="8" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="296" spans="1:10" x14ac:dyDescent="0.25">
@@ -7085,7 +7093,7 @@
         <v>1</v>
       </c>
       <c r="J296" s="11" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="297" spans="1:10" x14ac:dyDescent="0.25">
@@ -7105,15 +7113,15 @@
         <v>1</v>
       </c>
       <c r="J297" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="298" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
+        <v>537</v>
+      </c>
+      <c r="B298" s="3" t="s">
         <v>538</v>
-      </c>
-      <c r="B298" s="3" t="s">
-        <v>539</v>
       </c>
       <c r="C298" s="1">
         <v>1971</v>
@@ -7122,7 +7130,7 @@
         <v>0</v>
       </c>
       <c r="J298" s="13" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="299" spans="1:10" x14ac:dyDescent="0.25">
@@ -7138,6 +7146,9 @@
       <c r="E299" s="1" t="b">
         <v>0</v>
       </c>
+      <c r="J299" s="14" t="s">
+        <v>672</v>
+      </c>
     </row>
     <row r="300" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
@@ -7169,10 +7180,10 @@
     </row>
     <row r="302" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
+        <v>553</v>
+      </c>
+      <c r="B302" s="3" t="s">
         <v>554</v>
-      </c>
-      <c r="B302" s="3" t="s">
-        <v>555</v>
       </c>
       <c r="C302" s="1">
         <v>1977</v>
@@ -7183,10 +7194,10 @@
     </row>
     <row r="303" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
+        <v>567</v>
+      </c>
+      <c r="B303" s="3" t="s">
         <v>568</v>
-      </c>
-      <c r="B303" s="3" t="s">
-        <v>569</v>
       </c>
       <c r="C303" s="1">
         <v>2005</v>
@@ -7197,10 +7208,10 @@
     </row>
     <row r="304" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
+        <v>661</v>
+      </c>
+      <c r="B304" s="3" t="s">
         <v>662</v>
-      </c>
-      <c r="B304" s="3" t="s">
-        <v>663</v>
       </c>
       <c r="C304" s="1">
         <v>1998</v>
@@ -7228,10 +7239,10 @@
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
+        <v>632</v>
+      </c>
+      <c r="B306" s="3" t="s">
         <v>633</v>
-      </c>
-      <c r="B306" s="3" t="s">
-        <v>634</v>
       </c>
       <c r="C306" s="1">
         <v>1995</v>
@@ -7380,10 +7391,10 @@
     </row>
     <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
+        <v>663</v>
+      </c>
+      <c r="B316" s="3" t="s">
         <v>664</v>
-      </c>
-      <c r="B316" s="3" t="s">
-        <v>665</v>
       </c>
       <c r="C316" s="1">
         <v>1995</v>
@@ -7394,10 +7405,10 @@
     </row>
     <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
+        <v>500</v>
+      </c>
+      <c r="B317" s="3" t="s">
         <v>501</v>
-      </c>
-      <c r="B317" s="3" t="s">
-        <v>502</v>
       </c>
       <c r="C317" s="1">
         <v>1994</v>
@@ -7425,10 +7436,10 @@
     </row>
     <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
+        <v>525</v>
+      </c>
+      <c r="B319" s="3" t="s">
         <v>526</v>
-      </c>
-      <c r="B319" s="3" t="s">
-        <v>527</v>
       </c>
       <c r="C319" s="1">
         <v>1995</v>
@@ -7515,10 +7526,10 @@
     </row>
     <row r="325" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
+        <v>665</v>
+      </c>
+      <c r="B325" s="3" t="s">
         <v>666</v>
-      </c>
-      <c r="B325" s="3" t="s">
-        <v>667</v>
       </c>
       <c r="C325" s="1">
         <v>2017</v>
@@ -7591,11 +7602,14 @@
       <c r="E329" s="11" t="b">
         <v>1</v>
       </c>
+      <c r="J329" s="1" t="s">
+        <v>492</v>
+      </c>
     </row>
     <row r="330" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J330" s="10">
         <f>SUM(F2:F330)</f>
-        <v>12050</v>
+        <v>12150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>